<commit_message>
Update .env, README, and workbook
</commit_message>
<xml_diff>
--- a/test-datafile-with formula.xlsx
+++ b/test-datafile-with formula.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vramasubbu\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\ExcelFileFormulaExtraction\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8F4C6B8D-9E27-4226-91DB-AAE377216A11}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B652AD53-3A4C-49F0-BADA-403B04109C59}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25180" windowHeight="16140" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1900" yWindow="1900" windowWidth="18720" windowHeight="11650" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Commissions" sheetId="1" r:id="rId1"/>
@@ -39,10 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="152" uniqueCount="53">
-  <si>
-    <t>Central Sierra Insurance</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="151" uniqueCount="52">
   <si>
     <t>First Name</t>
   </si>
@@ -185,20 +182,20 @@
     <t>Mode</t>
   </si>
   <si>
-    <t>Central Sierra Insurance
+    <t>Commission_Level</t>
+  </si>
+  <si>
+    <t>Bonus_Rate</t>
+  </si>
+  <si>
+    <t>Tables!$A$2:$A$6</t>
+  </si>
+  <si>
+    <t>Tables!$B$2:$B$6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
 Agent Commissions and Bonus Data</t>
-  </si>
-  <si>
-    <t>Commission_Level</t>
-  </si>
-  <si>
-    <t>Bonus_Rate</t>
-  </si>
-  <si>
-    <t>Tables!$A$2:$A$6</t>
-  </si>
-  <si>
-    <t>Tables!$B$2:$B$6</t>
   </si>
 </sst>
 </file>
@@ -613,6 +610,17 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="18" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="10" fontId="3" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="9" xfId="1" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="10" xfId="1" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="17" xfId="1" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="11" xfId="1" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="6" fontId="3" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment indent="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment indent="2"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="19" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -640,17 +648,6 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="10" fontId="3" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="9" xfId="1" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="10" xfId="1" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="17" xfId="1" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="11" xfId="1" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="6" fontId="3" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment indent="2"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment indent="2"/>
-    </xf>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -668,10 +665,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1004,46 +997,46 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A1" s="30" t="s">
-        <v>48</v>
-      </c>
-      <c r="B1" s="31"/>
-      <c r="C1" s="31"/>
-      <c r="D1" s="31"/>
-      <c r="E1" s="31"/>
-      <c r="F1" s="31"/>
-      <c r="G1" s="32"/>
+      <c r="A1" s="37" t="s">
+        <v>51</v>
+      </c>
+      <c r="B1" s="38"/>
+      <c r="C1" s="38"/>
+      <c r="D1" s="38"/>
+      <c r="E1" s="38"/>
+      <c r="F1" s="38"/>
+      <c r="G1" s="39"/>
     </row>
     <row r="2" spans="1:7" ht="43.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A2" s="33"/>
-      <c r="B2" s="34"/>
-      <c r="C2" s="34"/>
-      <c r="D2" s="34"/>
-      <c r="E2" s="34"/>
-      <c r="F2" s="34"/>
-      <c r="G2" s="35"/>
+      <c r="A2" s="40"/>
+      <c r="B2" s="41"/>
+      <c r="C2" s="41"/>
+      <c r="D2" s="41"/>
+      <c r="E2" s="41"/>
+      <c r="F2" s="41"/>
+      <c r="G2" s="42"/>
     </row>
     <row r="4" spans="1:7" ht="33" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="5" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B4" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="D4" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="C4" s="5" t="s">
-        <v>1</v>
-      </c>
-      <c r="D4" s="5" t="s">
+      <c r="E4" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="E4" s="5" t="s">
+      <c r="F4" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="F4" s="5" t="s">
-        <v>5</v>
-      </c>
       <c r="G4" s="11" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="5" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.35">
@@ -1051,19 +1044,19 @@
         <v>101</v>
       </c>
       <c r="B5" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="D5" s="3" t="s">
         <v>7</v>
-      </c>
-      <c r="C5" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="D5" s="3" t="s">
-        <v>8</v>
       </c>
       <c r="E5" s="4">
         <v>15000</v>
       </c>
-      <c r="F5" s="39">
-        <f>_xlfn.XLOOKUP(E5,Commission_Level,Bonus_Rate,,-1)</f>
+      <c r="F5" s="30">
+        <f t="shared" ref="F5:F14" si="0">_xlfn.XLOOKUP(E5,Commission_Level,Bonus_Rate,,-1)</f>
         <v>2.5000000000000001E-2</v>
       </c>
       <c r="G5" s="4">
@@ -1076,23 +1069,23 @@
         <v>102</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="E6" s="4">
         <v>12000</v>
       </c>
-      <c r="F6" s="39">
-        <f>_xlfn.XLOOKUP(E6,Commission_Level,Bonus_Rate,,-1)</f>
+      <c r="F6" s="30">
+        <f t="shared" si="0"/>
         <v>2.2499999999999999E-2</v>
       </c>
       <c r="G6" s="4">
-        <f t="shared" ref="G6:G14" si="0">E6+(E6*F6)</f>
+        <f t="shared" ref="G6:G14" si="1">E6+(E6*F6)</f>
         <v>12270</v>
       </c>
     </row>
@@ -1101,23 +1094,23 @@
         <v>103</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E7" s="4">
         <v>5500</v>
       </c>
-      <c r="F7" s="39">
-        <f>_xlfn.XLOOKUP(E7,Commission_Level,Bonus_Rate,,-1)</f>
+      <c r="F7" s="30">
+        <f t="shared" si="0"/>
         <v>1.4999999999999999E-2</v>
       </c>
       <c r="G7" s="4">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>5582.5</v>
       </c>
     </row>
@@ -1126,23 +1119,23 @@
         <v>104</v>
       </c>
       <c r="B8" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="D8" s="3" t="s">
         <v>14</v>
-      </c>
-      <c r="C8" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="D8" s="3" t="s">
-        <v>15</v>
       </c>
       <c r="E8" s="4">
         <v>4500</v>
       </c>
-      <c r="F8" s="39">
-        <f>_xlfn.XLOOKUP(E8,Commission_Level,Bonus_Rate,,-1)</f>
+      <c r="F8" s="30">
+        <f t="shared" si="0"/>
         <v>1.4999999999999999E-2</v>
       </c>
       <c r="G8" s="4">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>4567.5</v>
       </c>
     </row>
@@ -1151,23 +1144,23 @@
         <v>105</v>
       </c>
       <c r="B9" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="D9" s="3" t="s">
         <v>17</v>
-      </c>
-      <c r="C9" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="D9" s="3" t="s">
-        <v>18</v>
       </c>
       <c r="E9" s="4">
         <v>3000</v>
       </c>
-      <c r="F9" s="39">
-        <f>_xlfn.XLOOKUP(E9,Commission_Level,Bonus_Rate,,-1)</f>
+      <c r="F9" s="30">
+        <f t="shared" si="0"/>
         <v>1.4999999999999999E-2</v>
       </c>
       <c r="G9" s="4">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>3045</v>
       </c>
     </row>
@@ -1176,23 +1169,23 @@
         <v>115</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E10" s="4">
         <v>3000</v>
       </c>
-      <c r="F10" s="39">
-        <f>_xlfn.XLOOKUP(E10,Commission_Level,Bonus_Rate,,-1)</f>
+      <c r="F10" s="30">
+        <f t="shared" si="0"/>
         <v>1.4999999999999999E-2</v>
       </c>
       <c r="G10" s="4">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>3045</v>
       </c>
     </row>
@@ -1201,23 +1194,23 @@
         <v>117</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D11" s="3" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="E11" s="4">
         <v>4700</v>
       </c>
-      <c r="F11" s="39">
-        <f>_xlfn.XLOOKUP(E11,Commission_Level,Bonus_Rate,,-1)</f>
+      <c r="F11" s="30">
+        <f t="shared" si="0"/>
         <v>1.4999999999999999E-2</v>
       </c>
       <c r="G11" s="4">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>4770.5</v>
       </c>
     </row>
@@ -1226,23 +1219,23 @@
         <v>119</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="E12" s="4">
         <v>4000</v>
       </c>
-      <c r="F12" s="39">
-        <f>_xlfn.XLOOKUP(E12,Commission_Level,Bonus_Rate,,-1)</f>
+      <c r="F12" s="30">
+        <f t="shared" si="0"/>
         <v>1.4999999999999999E-2</v>
       </c>
       <c r="G12" s="4">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>4060</v>
       </c>
     </row>
@@ -1251,23 +1244,23 @@
         <v>120</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D13" s="3" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E13" s="4">
         <v>4000</v>
       </c>
-      <c r="F13" s="39">
-        <f>_xlfn.XLOOKUP(E13,Commission_Level,Bonus_Rate,,-1)</f>
+      <c r="F13" s="30">
+        <f t="shared" si="0"/>
         <v>1.4999999999999999E-2</v>
       </c>
       <c r="G13" s="4">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>4060</v>
       </c>
     </row>
@@ -1276,69 +1269,69 @@
         <v>125</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="D14" s="3" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E14" s="4">
         <v>12000</v>
       </c>
-      <c r="F14" s="39">
-        <f>_xlfn.XLOOKUP(E14,Commission_Level,Bonus_Rate,,-1)</f>
+      <c r="F14" s="30">
+        <f t="shared" si="0"/>
         <v>2.2499999999999999E-2</v>
       </c>
       <c r="G14" s="4">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>12270</v>
       </c>
     </row>
     <row r="17" spans="3:5" ht="20.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="C17" s="36" t="s">
-        <v>33</v>
-      </c>
-      <c r="D17" s="37"/>
-      <c r="E17" s="38"/>
+      <c r="C17" s="43" t="s">
+        <v>32</v>
+      </c>
+      <c r="D17" s="44"/>
+      <c r="E17" s="45"/>
     </row>
     <row r="18" spans="3:5" ht="20.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C18" s="6" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D18" s="7"/>
-      <c r="E18" s="40">
+      <c r="E18" s="31">
         <f>SUMIF($D$5:$D$14,C18,$G$5:$G$14)</f>
         <v>40332.5</v>
       </c>
     </row>
     <row r="19" spans="3:5" ht="20.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C19" s="8" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D19" s="9"/>
-      <c r="E19" s="41">
-        <f t="shared" ref="E19:E20" si="1">SUMIF($D$5:$D$14,C19,$G$5:$G$14)</f>
+      <c r="E19" s="32">
+        <f t="shared" ref="E19:E20" si="2">SUMIF($D$5:$D$14,C19,$G$5:$G$14)</f>
         <v>15315</v>
       </c>
     </row>
     <row r="20" spans="3:5" ht="20.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C20" s="8" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D20" s="9"/>
-      <c r="E20" s="41">
-        <f t="shared" si="1"/>
+      <c r="E20" s="32">
+        <f t="shared" si="2"/>
         <v>13398</v>
       </c>
     </row>
     <row r="21" spans="3:5" ht="20.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C21" s="8"/>
       <c r="D21" s="29" t="s">
-        <v>30</v>
-      </c>
-      <c r="E21" s="42">
+        <v>29</v>
+      </c>
+      <c r="E21" s="33">
         <f>SUM(E18:E20)</f>
         <v>69045.5</v>
       </c>
@@ -1346,9 +1339,9 @@
     <row r="22" spans="3:5" ht="20.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C22" s="8"/>
       <c r="D22" s="29" t="s">
-        <v>46</v>
-      </c>
-      <c r="E22" s="42">
+        <v>45</v>
+      </c>
+      <c r="E22" s="33">
         <f>AVERAGE(G5:G14)</f>
         <v>6904.55</v>
       </c>
@@ -1356,9 +1349,9 @@
     <row r="23" spans="3:5" ht="20.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C23" s="8"/>
       <c r="D23" s="29" t="s">
-        <v>47</v>
-      </c>
-      <c r="E23" s="42">
+        <v>46</v>
+      </c>
+      <c r="E23" s="33">
         <f>_xlfn.MODE.SNGL(G5:G14)</f>
         <v>12270</v>
       </c>
@@ -1366,9 +1359,9 @@
     <row r="24" spans="3:5" ht="20.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C24" s="24"/>
       <c r="D24" s="28" t="s">
-        <v>45</v>
-      </c>
-      <c r="E24" s="43">
+        <v>44</v>
+      </c>
+      <c r="E24" s="34">
         <f>MEDIAN(G5:G14)</f>
         <v>4669</v>
       </c>
@@ -1406,9 +1399,7 @@
       <c r="F1" s="17"/>
     </row>
     <row r="2" spans="1:6" ht="23.5" x14ac:dyDescent="0.55000000000000004">
-      <c r="A2" s="18" t="s">
-        <v>0</v>
-      </c>
+      <c r="A2" s="18"/>
       <c r="B2" s="19"/>
       <c r="C2" s="19"/>
       <c r="D2" s="19"/>
@@ -1417,7 +1408,7 @@
     </row>
     <row r="3" spans="1:6" ht="23.5" x14ac:dyDescent="0.55000000000000004">
       <c r="A3" s="18" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B3" s="19"/>
       <c r="C3" s="19"/>
@@ -1443,22 +1434,22 @@
     </row>
     <row r="6" spans="1:6" ht="32.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B6" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="D6" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="C6" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="D6" s="2" t="s">
-        <v>3</v>
-      </c>
       <c r="E6" s="2" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="F6" s="10" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="7" spans="1:6" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.35">
@@ -1466,18 +1457,18 @@
         <v>101</v>
       </c>
       <c r="B7" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="D7" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="C7" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="D7" s="3" t="s">
-        <v>8</v>
-      </c>
       <c r="E7" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="F7" s="44" t="str">
+        <v>34</v>
+      </c>
+      <c r="F7" s="35" t="str">
         <f>IF(E7="Business Policy","No","Yes")</f>
         <v>Yes</v>
       </c>
@@ -1487,18 +1478,18 @@
         <v>102</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="E8" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="F8" s="45" t="str">
+        <v>38</v>
+      </c>
+      <c r="F8" s="36" t="str">
         <f t="shared" ref="F8:F27" si="0">IF(E8="Business Policy","No","Yes")</f>
         <v>No</v>
       </c>
@@ -1508,18 +1499,18 @@
         <v>103</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E9" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="F9" s="45" t="str">
+        <v>39</v>
+      </c>
+      <c r="F9" s="36" t="str">
         <f t="shared" si="0"/>
         <v>Yes</v>
       </c>
@@ -1529,18 +1520,18 @@
         <v>104</v>
       </c>
       <c r="B10" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C10" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="D10" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="C10" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="D10" s="3" t="s">
-        <v>15</v>
-      </c>
       <c r="E10" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="F10" s="45" t="str">
+        <v>36</v>
+      </c>
+      <c r="F10" s="36" t="str">
         <f t="shared" si="0"/>
         <v>Yes</v>
       </c>
@@ -1550,18 +1541,18 @@
         <v>105</v>
       </c>
       <c r="B11" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C11" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="D11" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="C11" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="D11" s="3" t="s">
-        <v>18</v>
-      </c>
       <c r="E11" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="F11" s="45" t="str">
+        <v>35</v>
+      </c>
+      <c r="F11" s="36" t="str">
         <f t="shared" si="0"/>
         <v>Yes</v>
       </c>
@@ -1571,18 +1562,18 @@
         <v>115</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E12" s="3" t="s">
-        <v>38</v>
-      </c>
-      <c r="F12" s="45" t="str">
+        <v>37</v>
+      </c>
+      <c r="F12" s="36" t="str">
         <f t="shared" si="0"/>
         <v>Yes</v>
       </c>
@@ -1592,18 +1583,18 @@
         <v>117</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D13" s="3" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="E13" s="3" t="s">
-        <v>38</v>
-      </c>
-      <c r="F13" s="45" t="str">
+        <v>37</v>
+      </c>
+      <c r="F13" s="36" t="str">
         <f t="shared" si="0"/>
         <v>Yes</v>
       </c>
@@ -1613,18 +1604,18 @@
         <v>119</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D14" s="3" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="E14" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="F14" s="45" t="str">
+        <v>34</v>
+      </c>
+      <c r="F14" s="36" t="str">
         <f t="shared" si="0"/>
         <v>Yes</v>
       </c>
@@ -1634,18 +1625,18 @@
         <v>120</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C15" s="3" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D15" s="3" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E15" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="F15" s="45" t="str">
+        <v>38</v>
+      </c>
+      <c r="F15" s="36" t="str">
         <f t="shared" si="0"/>
         <v>No</v>
       </c>
@@ -1655,18 +1646,18 @@
         <v>125</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C16" s="3" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="D16" s="3" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E16" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="F16" s="45" t="str">
+        <v>39</v>
+      </c>
+      <c r="F16" s="36" t="str">
         <f t="shared" si="0"/>
         <v>Yes</v>
       </c>
@@ -1676,18 +1667,18 @@
         <v>102</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C17" s="3" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D17" s="3" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="E17" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="F17" s="45" t="str">
+        <v>36</v>
+      </c>
+      <c r="F17" s="36" t="str">
         <f t="shared" si="0"/>
         <v>Yes</v>
       </c>
@@ -1697,18 +1688,18 @@
         <v>103</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C18" s="3" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D18" s="3" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E18" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="F18" s="45" t="str">
+        <v>35</v>
+      </c>
+      <c r="F18" s="36" t="str">
         <f t="shared" si="0"/>
         <v>Yes</v>
       </c>
@@ -1718,18 +1709,18 @@
         <v>117</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C19" s="3" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D19" s="3" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="E19" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="F19" s="45" t="str">
+        <v>38</v>
+      </c>
+      <c r="F19" s="36" t="str">
         <f t="shared" si="0"/>
         <v>No</v>
       </c>
@@ -1739,18 +1730,18 @@
         <v>104</v>
       </c>
       <c r="B20" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C20" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="D20" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="C20" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="D20" s="3" t="s">
-        <v>15</v>
-      </c>
       <c r="E20" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="F20" s="45" t="str">
+        <v>39</v>
+      </c>
+      <c r="F20" s="36" t="str">
         <f t="shared" si="0"/>
         <v>Yes</v>
       </c>
@@ -1760,18 +1751,18 @@
         <v>105</v>
       </c>
       <c r="B21" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C21" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="D21" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="C21" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="D21" s="3" t="s">
-        <v>18</v>
-      </c>
       <c r="E21" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="F21" s="45" t="str">
+        <v>36</v>
+      </c>
+      <c r="F21" s="36" t="str">
         <f t="shared" si="0"/>
         <v>Yes</v>
       </c>
@@ -1781,18 +1772,18 @@
         <v>105</v>
       </c>
       <c r="B22" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C22" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="D22" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="C22" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="D22" s="3" t="s">
-        <v>18</v>
-      </c>
       <c r="E22" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="F22" s="45" t="str">
+        <v>34</v>
+      </c>
+      <c r="F22" s="36" t="str">
         <f t="shared" si="0"/>
         <v>Yes</v>
       </c>
@@ -1802,18 +1793,18 @@
         <v>115</v>
       </c>
       <c r="B23" s="3" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C23" s="3" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D23" s="3" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E23" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="F23" s="45" t="str">
+        <v>35</v>
+      </c>
+      <c r="F23" s="36" t="str">
         <f t="shared" si="0"/>
         <v>Yes</v>
       </c>
@@ -1823,18 +1814,18 @@
         <v>102</v>
       </c>
       <c r="B24" s="3" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C24" s="3" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D24" s="3" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="E24" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="F24" s="45" t="str">
+        <v>38</v>
+      </c>
+      <c r="F24" s="36" t="str">
         <f t="shared" si="0"/>
         <v>No</v>
       </c>
@@ -1844,18 +1835,18 @@
         <v>103</v>
       </c>
       <c r="B25" s="3" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C25" s="3" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D25" s="3" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E25" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="F25" s="45" t="str">
+        <v>39</v>
+      </c>
+      <c r="F25" s="36" t="str">
         <f t="shared" si="0"/>
         <v>Yes</v>
       </c>
@@ -1865,18 +1856,18 @@
         <v>104</v>
       </c>
       <c r="B26" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C26" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="D26" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="C26" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="D26" s="3" t="s">
-        <v>15</v>
-      </c>
       <c r="E26" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="F26" s="45" t="str">
+        <v>36</v>
+      </c>
+      <c r="F26" s="36" t="str">
         <f t="shared" si="0"/>
         <v>Yes</v>
       </c>
@@ -1886,18 +1877,18 @@
         <v>105</v>
       </c>
       <c r="B27" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C27" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="D27" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="C27" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="D27" s="3" t="s">
-        <v>18</v>
-      </c>
       <c r="E27" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="F27" s="45" t="str">
+        <v>38</v>
+      </c>
+      <c r="F27" s="36" t="str">
         <f t="shared" si="0"/>
         <v>No</v>
       </c>
@@ -1926,13 +1917,13 @@
   <sheetData>
     <row r="1" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="27" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B1" s="13" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D1" s="13" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="2" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.35">
@@ -2009,7 +2000,7 @@
     </row>
     <row r="9" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" s="12" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="D9" s="3" t="str">
         <f>_xlfn.CONCAT(Commissions!C12," ",Commissions!B12,", ",Commissions!D12)</f>
@@ -2018,7 +2009,7 @@
     </row>
     <row r="10" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A10" s="3" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="D10" s="3" t="str">
         <f>_xlfn.CONCAT(Commissions!C13," ",Commissions!B13,", ",Commissions!D13)</f>
@@ -2027,7 +2018,7 @@
     </row>
     <row r="11" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A11" s="3" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="D11" s="3" t="str">
         <f>_xlfn.CONCAT(Commissions!C14," ",Commissions!B14,", ",Commissions!D14)</f>
@@ -2036,34 +2027,34 @@
     </row>
     <row r="12" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A12" s="3" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="13" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A13" s="3" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D13" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="E13" s="1" t="s">
         <v>49</v>
-      </c>
-      <c r="E13" s="1" t="s">
-        <v>51</v>
       </c>
     </row>
     <row r="14" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A14" s="3" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="D14" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="E14" s="1" t="s">
         <v>50</v>
-      </c>
-      <c r="E14" s="1" t="s">
-        <v>52</v>
       </c>
     </row>
     <row r="15" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A15" s="3" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="16" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.35"/>
@@ -2094,6 +2085,19 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <Notes xmlns="d2abd38f-6d5a-473d-b1ba-4829743c656b" xsi:nil="true"/>
+    <Process xmlns="d2abd38f-6d5a-473d-b1ba-4829743c656b" xsi:nil="true"/>
+    <TaxCatchAll xmlns="59d4ac86-31f8-4cd3-8d96-c5f03de7de39" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="d2abd38f-6d5a-473d-b1ba-4829743c656b">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100461191214793DB46A34E2E7DB15AFA8E" ma:contentTypeVersion="15" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="5331cddcf6220ef1ddc3181d6a288a5b">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="d2abd38f-6d5a-473d-b1ba-4829743c656b" xmlns:ns3="59d4ac86-31f8-4cd3-8d96-c5f03de7de39" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="8eb064515aa35fd5aa3f9257aa49d970" ns2:_="" ns3:_="">
     <xsd:import namespace="d2abd38f-6d5a-473d-b1ba-4829743c656b"/>
@@ -2331,20 +2335,15 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <Notes xmlns="d2abd38f-6d5a-473d-b1ba-4829743c656b" xsi:nil="true"/>
-    <Process xmlns="d2abd38f-6d5a-473d-b1ba-4829743c656b" xsi:nil="true"/>
-    <TaxCatchAll xmlns="59d4ac86-31f8-4cd3-8d96-c5f03de7de39" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="d2abd38f-6d5a-473d-b1ba-4829743c656b">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<senna xmlns="http://customxml.org">
+  <kers>Hs6HMymbh7RjiGDJzMWlbXPlVJqMeqCGdjj507SZQ6U=</kers>
+  <massa>4/19/2026 10:04:21 PM</massa>
+  <hamilton>true</hamilton>
+</senna>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
@@ -2353,15 +2352,18 @@
 </FormTemplates>
 </file>
 
-<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
-<senna xmlns="http://customxml.org">
-  <kers>Hs6HMymbh7RjiGDJzMWlbXPlVJqMeqCGdjj507SZQ6U=</kers>
-  <massa>4/19/2026 10:04:21 PM</massa>
-  <hamilton>true</hamilton>
-</senna>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1EBE76BD-16FD-4778-96ED-D0906907A677}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="d2abd38f-6d5a-473d-b1ba-4829743c656b"/>
+    <ds:schemaRef ds:uri="59d4ac86-31f8-4cd3-8d96-c5f03de7de39"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F517133C-5F54-4ADE-A26E-5318B858363F}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2380,29 +2382,18 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1EBE76BD-16FD-4778-96ED-D0906907A677}">
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BAB07D4B-0B16-4F09-ABE9-B087D84E94DD}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="d2abd38f-6d5a-473d-b1ba-4829743c656b"/>
-    <ds:schemaRef ds:uri="59d4ac86-31f8-4cd3-8d96-c5f03de7de39"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8B9185AC-E8CD-448F-AD85-7CD1F9CB6815}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://customxml.org"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BAB07D4B-0B16-4F09-ABE9-B087D84E94DD}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8B9185AC-E8CD-448F-AD85-7CD1F9CB6815}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://customxml.org"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>